<commit_message>
Auto Update Lottery Data
</commit_message>
<xml_diff>
--- a/最新開獎紀錄.xlsx
+++ b/最新開獎紀錄.xlsx
@@ -2560,84 +2560,84 @@
     <row r="2" s="5">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>07/24(五)</t>
+          <t>07/25(六)</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>3  1  0  8</t>
+          <t>9  0  4  8</t>
         </is>
       </c>
     </row>
     <row r="3" s="5">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>07/25(六)</t>
+          <t>07/27(一)</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>9  0  4  8</t>
+          <t>5  9  1  0</t>
         </is>
       </c>
     </row>
     <row r="4" s="5">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>07/27(一)</t>
+          <t>07/28(二)</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>5  9  1  0</t>
+          <t>0  4  3  3</t>
         </is>
       </c>
     </row>
     <row r="5" s="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>07/28(二)</t>
+          <t>07/29(三)</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>0  4  3  3</t>
+          <t>7  6  8  5</t>
         </is>
       </c>
     </row>
     <row r="6" s="5">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>07/29(三)</t>
+          <t>07/30(四)</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>7  6  8  5</t>
+          <t>2  9  3  1</t>
         </is>
       </c>
     </row>
     <row r="7" s="5">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>07/30(四)</t>
+          <t>07/31(五)</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>2  9  3  1</t>
+          <t>7  1  9  8</t>
         </is>
       </c>
     </row>
     <row r="8" s="5">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>07/31(五)</t>
+          <t>08/01(六)</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>7  1  9  8</t>
+          <t>7  1  9  5</t>
         </is>
       </c>
       <c r="E8" s="4" t="n"/>
@@ -2645,36 +2645,36 @@
     <row r="9" s="5">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>08/01(六)</t>
+          <t>08/03(一)</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>7  1  9  5</t>
+          <t>6  0  1  6</t>
         </is>
       </c>
     </row>
     <row r="10" s="5">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>08/03(一)</t>
+          <t>08/04(二)</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>6  0  1  6</t>
+          <t>1  8  4  3</t>
         </is>
       </c>
     </row>
     <row r="11" s="5">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>08/04(二)</t>
+          <t>08/05(三)</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>1  8  4  3</t>
+          <t>0  8  2  3</t>
         </is>
       </c>
     </row>

</xml_diff>